<commit_message>
Week 6: Completed JMeter performance tests and generated reports
</commit_message>
<xml_diff>
--- a/results/Selenium_Final_Report.xlsx
+++ b/results/Selenium_Final_Report.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="185">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -557,6 +557,15 @@
   </si>
   <si>
     <t>Error: Password Mismatch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error: Alert Text: Backend </t>
+  </si>
+  <si>
+    <t>Error: argument of type 'No</t>
+  </si>
+  <si>
+    <t>FAIL</t>
   </si>
   <si>
     <t>PASS</t>
@@ -970,10 +979,10 @@
         <v>158</v>
       </c>
       <c r="G2" t="s">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="H2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -996,10 +1005,10 @@
         <v>159</v>
       </c>
       <c r="G3" t="s">
-        <v>159</v>
+        <v>181</v>
       </c>
       <c r="H3" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1022,10 +1031,10 @@
         <v>160</v>
       </c>
       <c r="G4" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="H4" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1051,7 +1060,7 @@
         <v>161</v>
       </c>
       <c r="H5" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1074,10 +1083,10 @@
         <v>162</v>
       </c>
       <c r="G6" t="s">
-        <v>162</v>
+        <v>181</v>
       </c>
       <c r="H6" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1100,10 +1109,10 @@
         <v>163</v>
       </c>
       <c r="G7" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="H7" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1126,10 +1135,10 @@
         <v>164</v>
       </c>
       <c r="G8" t="s">
-        <v>164</v>
+        <v>181</v>
       </c>
       <c r="H8" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1152,10 +1161,10 @@
         <v>165</v>
       </c>
       <c r="G9" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
       <c r="H9" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1178,10 +1187,10 @@
         <v>158</v>
       </c>
       <c r="G10" t="s">
-        <v>158</v>
+        <v>182</v>
       </c>
       <c r="H10" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1204,10 +1213,10 @@
         <v>166</v>
       </c>
       <c r="G11" t="s">
-        <v>166</v>
+        <v>181</v>
       </c>
       <c r="H11" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1230,10 +1239,10 @@
         <v>163</v>
       </c>
       <c r="G12" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="H12" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1256,10 +1265,10 @@
         <v>163</v>
       </c>
       <c r="G13" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="H13" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1282,10 +1291,10 @@
         <v>167</v>
       </c>
       <c r="G14" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="H14" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1308,10 +1317,10 @@
         <v>168</v>
       </c>
       <c r="G15" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="H15" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1334,10 +1343,10 @@
         <v>169</v>
       </c>
       <c r="G16" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="H16" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1360,10 +1369,10 @@
         <v>170</v>
       </c>
       <c r="G17" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="H17" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1389,7 +1398,7 @@
         <v>171</v>
       </c>
       <c r="H18" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1412,10 +1421,10 @@
         <v>158</v>
       </c>
       <c r="G19" t="s">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="H19" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1438,10 +1447,10 @@
         <v>172</v>
       </c>
       <c r="G20" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="H20" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1464,10 +1473,10 @@
         <v>158</v>
       </c>
       <c r="G21" t="s">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="H21" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1490,10 +1499,10 @@
         <v>173</v>
       </c>
       <c r="G22" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="H22" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1516,10 +1525,10 @@
         <v>174</v>
       </c>
       <c r="G23" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="H23" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1542,10 +1551,10 @@
         <v>175</v>
       </c>
       <c r="G24" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="H24" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1568,10 +1577,10 @@
         <v>175</v>
       </c>
       <c r="G25" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="H25" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1594,10 +1603,10 @@
         <v>176</v>
       </c>
       <c r="G26" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="H26" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1620,10 +1629,10 @@
         <v>177</v>
       </c>
       <c r="G27" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="H27" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1646,10 +1655,10 @@
         <v>178</v>
       </c>
       <c r="G28" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="H28" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1672,10 +1681,10 @@
         <v>179</v>
       </c>
       <c r="G29" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="H29" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1698,10 +1707,10 @@
         <v>180</v>
       </c>
       <c r="G30" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H30" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1724,10 +1733,10 @@
         <v>158</v>
       </c>
       <c r="G31" t="s">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="H31" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>